<commit_message>
Atualizacao automatica das notas
</commit_message>
<xml_diff>
--- a/Painel_Academico_PUCPR.xlsx
+++ b/Painel_Academico_PUCPR.xlsx
@@ -1938,13 +1938,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1960,12 +1962,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Maximo</t>
+          <t>Maximo Atual</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Media (%)</t>
+          <t>Pontos Pendentes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Media Atual (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Projecao Final (%)</t>
         </is>
       </c>
     </row>
@@ -1982,70 +1994,56 @@
         <v>20</v>
       </c>
       <c r="D2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E2" t="n">
+        <v>95</v>
+      </c>
+      <c r="F2" t="n">
         <v>95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Experiencia Criativa</t>
+          <t>Raciocinio Algoritmico</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52.8</v>
+        <v>18.11</v>
       </c>
       <c r="C3" t="n">
-        <v>110</v>
+        <v>32.5</v>
       </c>
       <c r="D3" t="n">
-        <v>48</v>
+        <v>10</v>
+      </c>
+      <c r="E3" t="n">
+        <v>55.72</v>
+      </c>
+      <c r="F3" t="n">
+        <v>55.72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Filosofia</t>
+          <t>Fundamentos Sistemas Ciberfisicos</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>61.4</v>
       </c>
       <c r="C4" t="n">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="D4" t="n">
-        <v>65.70999999999999</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Raciocinio Algoritmico</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>18.11</v>
-      </c>
-      <c r="C5" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>55.72</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Fundamentos Sistemas Ciberfisicos</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>61.4</v>
-      </c>
-      <c r="C6" t="n">
-        <v>123</v>
-      </c>
-      <c r="D6" t="n">
+        <v>467</v>
+      </c>
+      <c r="E4" t="n">
+        <v>49.92</v>
+      </c>
+      <c r="F4" t="n">
         <v>49.92</v>
       </c>
     </row>

</xml_diff>